<commit_message>
ScoresPossibles.xlsx : toujours montrer les 3 boules, ratées comprises
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012kwvW6KkNjDv7n8spegKrg
</commit_message>
<xml_diff>
--- a/ScoresPossibles.xlsx
+++ b/ScoresPossibles.xlsx
@@ -2853,6 +2853,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Chaque ligne compte les 3 boules : 0, 1, 2 ou 3 boules peuvent rater (0 point chacune).</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2861,7 +2868,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Façons de l'obtenir (boules dans les trous ; les autres boules ratées = 0)</t>
+          <t>Façons de l'obtenir avec les 3 boules (ratée = boule dans aucun trou, 0 point)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -2881,12 +2888,12 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>−5, −5</t>
+          <t>−5, −5, ratée</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>−5 − 5</t>
+          <t>−5 − 5 + 0</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2901,12 +2908,12 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>−5</t>
+          <t>−5, ratée, ratée</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>−5</t>
+          <t>−5 + 0 + 0</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2963,13 +2970,13 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>3 boules ratées
+          <t>ratée, ratée, ratée
 ♥, −5, −5</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>0
+          <t>0 + 0 + 0
 10 − 5 − 5</t>
         </is>
       </c>
@@ -2985,12 +2992,12 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>♣, −5</t>
+          <t>♣, −5, ratée</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>6 − 5</t>
+          <t>6 − 5 + 0</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -3005,14 +3012,14 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>♦, −5
-♠, −5</t>
+          <t>♦, −5, ratée
+♠, −5, ratée</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>8 − 5
-8 − 5</t>
+          <t>8 − 5 + 0
+8 − 5 + 0</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -3027,13 +3034,13 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>♥, −5
+          <t>♥, −5, ratée
 15, −5, −5</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>10 − 5
+          <t>10 − 5 + 0
 15 − 5 − 5</t>
         </is>
       </c>
@@ -3049,12 +3056,12 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>♣</t>
+          <t>♣, ratée, ratée</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6 + 0 + 0</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -3089,14 +3096,14 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>♦
-♠</t>
+          <t>♦, ratée, ratée
+♠, ratée, ratée</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>8
-8</t>
+          <t>8 + 0 + 0
+8 + 0 + 0</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -3133,14 +3140,14 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>♥
-15, −5</t>
+          <t>♥, ratée, ratée
+15, −5, ratée</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>10
-15 − 5</t>
+          <t>10 + 0 + 0
+15 − 5 + 0</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -3181,12 +3188,12 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>♣, ♣</t>
+          <t>♣, ♣, ratée</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>6 + 6</t>
+          <t>6 + 6 + 0</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -3223,14 +3230,14 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>♦, ♣
-♣, ♠</t>
+          <t>♦, ♣, ratée
+♣, ♠, ratée</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>8 + 6
-6 + 8</t>
+          <t>8 + 6 + 0
+6 + 8 + 0</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -3245,13 +3252,13 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>15
+          <t>15, ratée, ratée
 ♥, ♥, −5</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>15
+          <t>15 + 0 + 0
 10 + 10 − 5</t>
         </is>
       </c>
@@ -3267,19 +3274,19 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>♥, ♣
-♦, ♦
-♦, ♠
-♠, ♠
+          <t>♥, ♣, ratée
+♦, ♦, ratée
+♦, ♠, ratée
+♠, ♠, ratée
 15, ♣, −5</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>10 + 6
-8 + 8
-8 + 8
-8 + 8
+          <t>10 + 6 + 0
+8 + 8 + 0
+8 + 8 + 0
+8 + 8 + 0
 15 + 6 − 5</t>
         </is>
       </c>
@@ -3295,16 +3302,16 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>♥, ♦
-♥, ♠
+          <t>♥, ♦, ratée
+♥, ♠, ratée
 15, ♦, −5
 15, ♠, −5</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>10 + 8
-10 + 8
+          <t>10 + 8 + 0
+10 + 8 + 0
 15 + 8 − 5
 15 + 8 − 5</t>
         </is>
@@ -3321,7 +3328,7 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>♥, ♥
+          <t>♥, ♥, ratée
 15, ♥, −5
 ♦, ♣, ♣
 ♣, ♣, ♠</t>
@@ -3329,7 +3336,7 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>10 + 10
+          <t>10 + 10 + 0
 15 + 10 − 5
 8 + 6 + 6
 6 + 6 + 8</t>
@@ -3347,12 +3354,12 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>15, ♣</t>
+          <t>15, ♣, ratée</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>15 + 6</t>
+          <t>15 + 6 + 0</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -3393,14 +3400,14 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>15, ♦
-15, ♠</t>
+          <t>15, ♦, ratée
+15, ♠, ratée</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>15 + 8
-15 + 8</t>
+          <t>15 + 8 + 0
+15 + 8 + 0</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -3441,12 +3448,12 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>15, ♥</t>
+          <t>15, ♥, ratée</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>15 + 10</t>
+          <t>15 + 10 + 0</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -3648,6 +3655,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Chaque ligne compte les 3 boules : 0, 1, 2 ou 3 boules peuvent rater (0 point chacune).</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3656,7 +3670,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Façons de l'obtenir (boules dans les trous ; les autres boules ratées = 0)</t>
+          <t>Façons de l'obtenir avec les 3 boules (ratée = boule dans aucun trou, 0 point)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -3676,12 +3690,12 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>−5, −5</t>
+          <t>−5, −5, ratée</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>−5 − 5</t>
+          <t>−5 − 5 + 0</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -3716,12 +3730,12 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>−5</t>
+          <t>−5, ratée, ratée</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>−5</t>
+          <t>−5 + 0 + 0</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -3756,12 +3770,12 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>♠, −5</t>
+          <t>♠, −5, ratée</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>4 − 5</t>
+          <t>4 − 5 + 0</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -3776,13 +3790,13 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>3 boules ratées
+          <t>ratée, ratée, ratée
 ♥, −5, −5</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>0
+          <t>0 + 0 + 0
 10 − 5 − 5</t>
         </is>
       </c>
@@ -3818,13 +3832,13 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>♦, −5
+          <t>♦, −5, ratée
 ♠, ♠, −5</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>8 − 5
+          <t>8 − 5 + 0
 4 + 4 − 5</t>
         </is>
       </c>
@@ -3840,12 +3854,12 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>♠</t>
+          <t>♠, ratée, ratée</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4 + 0 + 0</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -3860,13 +3874,13 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>♥, −5
+          <t>♥, −5, ratée
 15, −5, −5</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>10 − 5
+          <t>10 − 5 + 0
 15 − 5 − 5</t>
         </is>
       </c>
@@ -3882,13 +3896,13 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>♣, −5
+          <t>♣, −5, ratée
 ♦, ♠, −5</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>12 − 5
+          <t>12 − 5 + 0
 8 + 4 − 5</t>
         </is>
       </c>
@@ -3904,14 +3918,14 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>♦
-♠, ♠</t>
+          <t>♦, ratée, ratée
+♠, ♠, ratée</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>8
-4 + 4</t>
+          <t>8 + 0 + 0
+4 + 4 + 0</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -3946,14 +3960,14 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>♥
-15, −5</t>
+          <t>♥, ratée, ratée
+15, −5, ratée</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>10
-15 − 5</t>
+          <t>10 + 0 + 0
+15 − 5 + 0</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -3990,14 +4004,14 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>♣
-♦, ♠</t>
+          <t>♣, ratée, ratée
+♦, ♠, ratée</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>12
-8 + 4</t>
+          <t>12 + 0 + 0
+8 + 4 + 0</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -4032,13 +4046,13 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>♥, ♠
+          <t>♥, ♠, ratée
 15, ♠, −5</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>10 + 4
+          <t>10 + 4 + 0
 15 + 4 − 5</t>
         </is>
       </c>
@@ -4054,14 +4068,14 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>15
+          <t>15, ratée, ratée
 ♥, ♥, −5
 ♦, ♣, −5</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>15
+          <t>15 + 0 + 0
 10 + 10 − 5
 8 + 12 − 5</t>
         </is>
@@ -4078,15 +4092,15 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>♦, ♦
-♣, ♠
+          <t>♦, ♦, ratée
+♣, ♠, ratée
 ♦, ♠, ♠</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>8 + 8
-12 + 4
+          <t>8 + 8 + 0
+12 + 4 + 0
 8 + 4 + 4</t>
         </is>
       </c>
@@ -4122,14 +4136,14 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>♥, ♦
+          <t>♥, ♦, ratée
 15, ♦, −5
 ♥, ♠, ♠</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>10 + 8
+          <t>10 + 8 + 0
 15 + 8 − 5
 10 + 4 + 4</t>
         </is>
@@ -4146,13 +4160,13 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>15, ♠
+          <t>15, ♠, ratée
 ♣, ♣, −5</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>15 + 4
+          <t>15 + 4 + 0
 12 + 12 − 5</t>
         </is>
       </c>
@@ -4168,8 +4182,8 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>♥, ♥
-♦, ♣
+          <t>♥, ♥, ratée
+♦, ♣, ratée
 15, ♥, −5
 ♦, ♦, ♠
 ♣, ♠, ♠</t>
@@ -4177,8 +4191,8 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>10 + 10
-8 + 12
+          <t>10 + 10 + 0
+8 + 12 + 0
 15 + 10 − 5
 8 + 8 + 4
 12 + 4 + 4</t>
@@ -4196,14 +4210,14 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>♥, ♣
+          <t>♥, ♣, ratée
 15, ♣, −5
 ♥, ♦, ♠</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>10 + 12
+          <t>10 + 12 + 0
 15 + 12 − 5
 10 + 8 + 4</t>
         </is>
@@ -4220,13 +4234,13 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>15, ♦
+          <t>15, ♦, ratée
 15, ♠, ♠</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>15 + 8
+          <t>15 + 8 + 0
 15 + 4 + 4</t>
         </is>
       </c>
@@ -4242,14 +4256,14 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>♣, ♣
+          <t>♣, ♣, ratée
 ♥, ♥, ♠
 ♦, ♣, ♠</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>12 + 12
+          <t>12 + 12 + 0
 10 + 10 + 4
 8 + 12 + 4</t>
         </is>
@@ -4266,12 +4280,12 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>15, ♥</t>
+          <t>15, ♥, ratée</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>15 + 10</t>
+          <t>15 + 10 + 0</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -4308,13 +4322,13 @@
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>15, ♣
+          <t>15, ♣, ratée
 15, ♦, ♠</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>15 + 12
+          <t>15 + 12 + 0
 15 + 8 + 4</t>
         </is>
       </c>
@@ -4569,6 +4583,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Chaque ligne compte les 3 boules : 0, 1, 2 ou 3 boules peuvent rater (0 point chacune).</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4577,7 +4598,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Façons de l'obtenir (boules dans les trous ; les autres boules ratées = 0)</t>
+          <t>Façons de l'obtenir avec les 3 boules (ratée = boule dans aucun trou, 0 point)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -4597,12 +4618,12 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>−5, −5</t>
+          <t>−5, −5, ratée</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>−5 − 5</t>
+          <t>−5 − 5 + 0</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -4637,12 +4658,12 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>−5</t>
+          <t>−5, ratée, ratée</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>−5</t>
+          <t>−5 + 0 + 0</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -4677,12 +4698,12 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>♠, −5</t>
+          <t>♠, −5, ratée</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>4 − 5</t>
+          <t>4 − 5 + 0</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -4697,13 +4718,13 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>3 boules ratées
+          <t>ratée, ratée, ratée
 ♥, −5, −5</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>0
+          <t>0 + 0 + 0
 10 − 5 − 5</t>
         </is>
       </c>
@@ -4719,12 +4740,12 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>♣, −5</t>
+          <t>♣, −5, ratée</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>6 − 5</t>
+          <t>6 − 5 + 0</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -4759,12 +4780,12 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>♠</t>
+          <t>♠, ratée, ratée</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4 + 0 + 0</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -4779,14 +4800,14 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>♥, −5
+          <t>♥, −5, ratée
 15, −5, −5
 ♣, ♠, −5</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>10 − 5
+          <t>10 − 5 + 0
 15 − 5 − 5
 6 + 4 − 5</t>
         </is>
@@ -4803,13 +4824,13 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>♣
+          <t>♣, ratée, ratée
 ♦, −5, −5</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>6
+          <t>6 + 0 + 0
 16 − 5 − 5</t>
         </is>
       </c>
@@ -4845,12 +4866,12 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>♠, ♠</t>
+          <t>♠, ♠, ratée</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>4 + 4</t>
+          <t>4 + 4 + 0</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -4885,16 +4906,16 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>♥
-15, −5
-♣, ♠</t>
+          <t>♥, ratée, ratée
+15, −5, ratée
+♣, ♠, ratée</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>10
-15 − 5
-6 + 4</t>
+          <t>10 + 0 + 0
+15 − 5 + 0
+6 + 4 + 0</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -4909,13 +4930,13 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>♦, −5
+          <t>♦, −5, ratée
 ♥, ♣, −5</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>16 − 5
+          <t>16 − 5 + 0
 10 + 6 − 5</t>
         </is>
       </c>
@@ -4931,12 +4952,12 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>♣, ♣</t>
+          <t>♣, ♣, ratée</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>6 + 6</t>
+          <t>6 + 6 + 0</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -4951,14 +4972,14 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>♥, ♠
+          <t>♥, ♠, ratée
 15, ♠, −5
 ♣, ♠, ♠</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>10 + 4
+          <t>10 + 4 + 0
 15 + 4 − 5
 6 + 4 + 4</t>
         </is>
@@ -4975,14 +4996,14 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>15
+          <t>15, ratée, ratée
 ♥, ♥, −5
 ♦, ♠, −5</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>15
+          <t>15 + 0 + 0
 10 + 10 − 5
 16 + 4 − 5</t>
         </is>
@@ -4999,16 +5020,16 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>♦
-♥, ♣
+          <t>♦, ratée, ratée
+♥, ♣, ratée
 15, ♣, −5
 ♣, ♣, ♠</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>16
-10 + 6
+          <t>16 + 0 + 0
+10 + 6 + 0
 15 + 6 − 5
 6 + 6 + 4</t>
         </is>
@@ -5065,12 +5086,12 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>15, ♠</t>
+          <t>15, ♠, ratée</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>15 + 4</t>
+          <t>15 + 4 + 0</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -5085,16 +5106,16 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>♥, ♥
-♦, ♠
+          <t>♥, ♥, ratée
+♦, ♠, ratée
 15, ♥, −5
 ♥, ♣, ♠</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>10 + 10
-16 + 4
+          <t>10 + 10 + 0
+16 + 4 + 0
 15 + 10 − 5
 10 + 6 + 4</t>
         </is>
@@ -5111,13 +5132,13 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>15, ♣
+          <t>15, ♣, ratée
 ♥, ♦, −5</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>15 + 6
+          <t>15 + 6 + 0
 10 + 16 − 5</t>
         </is>
       </c>
@@ -5133,13 +5154,13 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>♦, ♣
+          <t>♦, ♣, ratée
 ♥, ♣, ♣</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>16 + 6
+          <t>16 + 6 + 0
 10 + 6 + 6</t>
         </is>
       </c>
@@ -5197,13 +5218,13 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>15, ♥
+          <t>15, ♥, ratée
 15, ♣, ♠</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>15 + 10
+          <t>15 + 10 + 0
 15 + 6 + 4</t>
         </is>
       </c>
@@ -5219,7 +5240,7 @@
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>♥, ♦
+          <t>♥, ♦, ratée
 15, ♦, −5
 ♥, ♥, ♣
 ♦, ♣, ♠</t>
@@ -5227,7 +5248,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>10 + 16
+          <t>10 + 16 + 0
 15 + 16 − 5
 10 + 10 + 6
 16 + 6 + 4</t>
@@ -5327,13 +5348,13 @@
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>15, ♦
+          <t>15, ♦, ratée
 15, ♥, ♣</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>15 + 16
+          <t>15 + 16 + 0
 15 + 10 + 6</t>
         </is>
       </c>
@@ -5349,13 +5370,13 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>♦, ♦
+          <t>♦, ♦, ratée
 ♥, ♦, ♣</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>16 + 16
+          <t>16 + 16 + 0
 10 + 16 + 6</t>
         </is>
       </c>
@@ -5544,6 +5565,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Chaque ligne compte les 3 boules : 0, 1, 2 ou 3 boules peuvent rater (0 point chacune).</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5552,7 +5580,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Façons de l'obtenir (boules dans les trous ; les autres boules ratées = 0)</t>
+          <t>Façons de l'obtenir avec les 3 boules (ratée = boule dans aucun trou, 0 point)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -5572,12 +5600,12 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>−5, −5</t>
+          <t>−5, −5, ratée</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>−5 − 5</t>
+          <t>−5 − 5 + 0</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -5612,12 +5640,12 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>−5</t>
+          <t>−5, ratée, ratée</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>−5</t>
+          <t>−5 + 0 + 0</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -5672,12 +5700,12 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>♠, −5</t>
+          <t>♠, −5, ratée</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>4 − 5</t>
+          <t>4 − 5 + 0</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -5692,12 +5720,12 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>3 boules ratées</t>
+          <t>ratée, ratée, ratée</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0 + 0 + 0</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -5712,12 +5740,12 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>♣, −5</t>
+          <t>♣, −5, ratée</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>6 − 5</t>
+          <t>6 − 5 + 0</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -5732,13 +5760,13 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>♦, −5
+          <t>♦, −5, ratée
 ♠, ♠, −5</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>8 − 5
+          <t>8 − 5 + 0
 4 + 4 − 5</t>
         </is>
       </c>
@@ -5754,12 +5782,12 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>♠</t>
+          <t>♠, ratée, ratée</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4 + 0 + 0</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -5796,12 +5824,12 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>♣</t>
+          <t>♣, ratée, ratée</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6 + 0 + 0</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -5838,14 +5866,14 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>♦
-♠, ♠</t>
+          <t>♦, ratée, ratée
+♠, ♠, ratée</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>8
-4 + 4</t>
+          <t>8 + 0 + 0
+4 + 4 + 0</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -5880,15 +5908,15 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>15, −5
-♣, ♠
+          <t>15, −5, ratée
+♣, ♠, ratée
 ♥, −5, −5</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>15 − 5
-6 + 4
+          <t>15 − 5 + 0
+6 + 4 + 0
 20 − 5 − 5</t>
         </is>
       </c>
@@ -5924,14 +5952,14 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>♦, ♠
-♣, ♣</t>
+          <t>♦, ♠, ratée
+♣, ♣, ratée</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>8 + 4
-6 + 6</t>
+          <t>8 + 4 + 0
+6 + 6 + 0</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -5946,14 +5974,14 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>♦, ♣
+          <t>♦, ♣, ratée
 15, ♠, −5
 ♣, ♠, ♠</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>8 + 6
+          <t>8 + 6 + 0
 15 + 4 − 5
 6 + 4 + 4</t>
         </is>
@@ -5970,14 +5998,14 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>15
-♥, −5</t>
+          <t>15, ratée, ratée
+♥, −5, ratée</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>15
-20 − 5</t>
+          <t>15 + 0 + 0
+20 − 5 + 0</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -5992,7 +6020,7 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>♦, ♦
+          <t>♦, ♦, ratée
 15, ♣, −5
 ♦, ♠, ♠
 ♣, ♣, ♠</t>
@@ -6000,7 +6028,7 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>8 + 8
+          <t>8 + 8 + 0
 15 + 6 − 5
 8 + 4 + 4
 6 + 6 + 4</t>
@@ -6040,13 +6068,13 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>15, ♠
+          <t>15, ♠, ratée
 ♥, ♠, −5</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>15 + 4
+          <t>15 + 4 + 0
 20 + 4 − 5</t>
         </is>
       </c>
@@ -6062,14 +6090,14 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>♥
+          <t>♥, ratée, ratée
 ♦, ♦, ♠
 ♦, ♣, ♣</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>20
+          <t>20 + 0 + 0
 8 + 8 + 4
 8 + 6 + 6</t>
         </is>
@@ -6086,13 +6114,13 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>15, ♣
+          <t>15, ♣, ratée
 ♥, ♣, −5</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>15 + 6
+          <t>15 + 6 + 0
 20 + 6 − 5</t>
         </is>
       </c>
@@ -6128,14 +6156,14 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>15, ♦
+          <t>15, ♦, ratée
 15, ♠, ♠
 ♥, ♦, −5</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>15 + 8
+          <t>15 + 8 + 0
 15 + 4 + 4
 20 + 8 − 5</t>
         </is>
@@ -6152,12 +6180,12 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>♥, ♠</t>
+          <t>♥, ♠, ratée</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>20 + 4</t>
+          <t>20 + 4 + 0</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -6192,12 +6220,12 @@
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>♥, ♣</t>
+          <t>♥, ♣, ratée</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>20 + 6</t>
+          <t>20 + 6 + 0</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -6234,13 +6262,13 @@
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>♥, ♦
+          <t>♥, ♦, ratée
 ♥, ♠, ♠</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>20 + 8
+          <t>20 + 8 + 0
 20 + 4 + 4</t>
         </is>
       </c>
@@ -6360,13 +6388,13 @@
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>15, ♥
+          <t>15, ♥, ratée
 ♥, ♥, −5</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>15 + 20
+          <t>15 + 20 + 0
 20 + 20 − 5</t>
         </is>
       </c>
@@ -6422,12 +6450,12 @@
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>♥, ♥</t>
+          <t>♥, ♥, ratée</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>20 + 20</t>
+          <t>20 + 20 + 0</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -6591,6 +6619,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Chaque ligne compte les 3 boules : 0, 1, 2 ou 3 boules peuvent rater (0 point chacune).</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -6599,7 +6634,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Façons de l'obtenir (boules dans les trous ; les autres boules ratées = 0)</t>
+          <t>Façons de l'obtenir avec les 3 boules (ratée = boule dans aucun trou, 0 point)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -6619,12 +6654,12 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>−5, −5</t>
+          <t>−5, −5, ratée</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>−10 − 10</t>
+          <t>−10 − 10 + 0</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -6659,12 +6694,12 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>−5</t>
+          <t>−5, ratée, ratée</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>−10</t>
+          <t>−10 + 0 + 0</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -6719,12 +6754,12 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>♠, −5</t>
+          <t>♠, −5, ratée</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>8 − 10</t>
+          <t>8 − 10 + 0</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -6739,13 +6774,13 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>3 boules ratées
+          <t>ratée, ratée, ratée
 ♥, −5, −5</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>0
+          <t>0 + 0 + 0
 20 − 10 − 10</t>
         </is>
       </c>
@@ -6761,12 +6796,12 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>♣, −5</t>
+          <t>♣, −5, ratée</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>12 − 10</t>
+          <t>12 − 10 + 0</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -6781,13 +6816,13 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>♦, −5
+          <t>♦, −5, ratée
 ♠, ♠, −5</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>16 − 10
+          <t>16 − 10 + 0
 8 + 8 − 10</t>
         </is>
       </c>
@@ -6803,12 +6838,12 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>♠</t>
+          <t>♠, ratée, ratée</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>8 + 0 + 0</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -6823,14 +6858,14 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>♥, −5
+          <t>♥, −5, ratée
 15, −5, −5
 ♣, ♠, −5</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>20 − 10
+          <t>20 − 10 + 0
 30 − 10 − 10
 12 + 8 − 10</t>
         </is>
@@ -6847,12 +6882,12 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>♣</t>
+          <t>♣, ratée, ratée</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12 + 0 + 0</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -6889,14 +6924,14 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>♦
-♠, ♠</t>
+          <t>♦, ratée, ratée
+♠, ♠, ratée</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>16
-8 + 8</t>
+          <t>16 + 0 + 0
+8 + 8 + 0</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -6933,16 +6968,16 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>♥
-15, −5
-♣, ♠</t>
+          <t>♥, ratée, ratée
+15, −5, ratée
+♣, ♠, ratée</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>20
-30 − 10
-12 + 8</t>
+          <t>20 + 0 + 0
+30 − 10 + 0
+12 + 8 + 0</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -6979,14 +7014,14 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>♦, ♠
-♣, ♣</t>
+          <t>♦, ♠, ratée
+♣, ♣, ratée</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>16 + 8
-12 + 12</t>
+          <t>16 + 8 + 0
+12 + 12 + 0</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -7021,16 +7056,16 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>♥, ♠
-♦, ♣
+          <t>♥, ♠, ratée
+♦, ♣, ratée
 15, ♠, −5
 ♣, ♠, ♠</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>20 + 8
-16 + 12
+          <t>20 + 8 + 0
+16 + 12 + 0
 30 + 8 − 10
 12 + 8 + 8</t>
         </is>
@@ -7047,13 +7082,13 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>15
+          <t>15, ratée, ratée
 ♥, ♥, −5</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>30
+          <t>30 + 0 + 0
 20 + 20 − 10</t>
         </is>
       </c>
@@ -7069,8 +7104,8 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>♥, ♣
-♦, ♦
+          <t>♥, ♣, ratée
+♦, ♦, ratée
 15, ♣, −5
 ♦, ♠, ♠
 ♣, ♣, ♠</t>
@@ -7078,8 +7113,8 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>20 + 12
-16 + 16
+          <t>20 + 12 + 0
+16 + 16 + 0
 30 + 12 − 10
 16 + 8 + 8
 12 + 12 + 8</t>
@@ -7097,7 +7132,7 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>♥, ♦
+          <t>♥, ♦, ratée
 15, ♦, −5
 ♥, ♠, ♠
 ♦, ♣, ♠</t>
@@ -7105,7 +7140,7 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>20 + 16
+          <t>20 + 16 + 0
 30 + 16 − 10
 20 + 8 + 8
 16 + 12 + 8</t>
@@ -7123,12 +7158,12 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>15, ♠</t>
+          <t>15, ♠, ratée</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>30 + 8</t>
+          <t>30 + 8 + 0</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -7143,7 +7178,7 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>♥, ♥
+          <t>♥, ♥, ratée
 15, ♥, −5
 ♥, ♣, ♠
 ♦, ♦, ♠
@@ -7152,7 +7187,7 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>20 + 20
+          <t>20 + 20 + 0
 30 + 20 − 10
 20 + 12 + 8
 16 + 16 + 8
@@ -7171,12 +7206,12 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>15, ♣</t>
+          <t>15, ♣, ratée</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>30 + 12</t>
+          <t>30 + 12 + 0</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -7215,13 +7250,13 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>15, ♦
+          <t>15, ♦, ratée
 15, ♠, ♠</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>30 + 16
+          <t>30 + 16 + 0
 30 + 8 + 8</t>
         </is>
       </c>
@@ -7259,13 +7294,13 @@
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>15, ♥
+          <t>15, ♥, ratée
 15, ♣, ♠</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>30 + 20
+          <t>30 + 20 + 0
 30 + 12 + 8</t>
         </is>
       </c>

</xml_diff>